<commit_message>
Add error handling and validation to Excel upgrade script
Co-authored-by: lancejlene-oss <240118005+lancejlene-oss@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/templates/worksheet.xlsx
+++ b/templates/worksheet.xlsx
@@ -401,6 +401,34 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3333750" cy="2857500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -425,6 +453,34 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3333750" cy="3333750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -461,6 +517,34 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3333750" cy="2962275"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -485,6 +569,34 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3333750" cy="2752725"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -521,6 +633,34 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3333750" cy="2857500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -545,6 +685,34 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3333750" cy="2543175"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1148,7 +1316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1285,109 +1453,118 @@
     </row>
     <row r="16"/>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+      <c r="A17" s="29" t="inlineStr">
+        <is>
+          <t>STEP 0 — PLAN SETUP &amp; ORIENTATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="30" t="inlineStr">
+        <is>
+          <t>INSTRUCTIONS:</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="31" t="inlineStr">
+        <is>
+          <t>1. Verify you have the LATEST REVISION of the plan set</t>
+        </is>
+      </c>
+      <c r="E19" s="32" t="inlineStr">
+        <is>
+          <t>☐ Latest revision confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="31" t="inlineStr">
+        <is>
+          <t>2. Check the scale on the title block (usually 1/4" = 1'-0")</t>
+        </is>
+      </c>
+      <c r="E20" s="32" t="inlineStr">
+        <is>
+          <t>☐ Scale verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="31" t="inlineStr">
+        <is>
+          <t>3. Verify scale by measuring a known dimension with your scale ruler</t>
+        </is>
+      </c>
+      <c r="E21" s="32" t="inlineStr">
+        <is>
+          <t>☐ Windstorm/code notes checked</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="31" t="inlineStr">
+        <is>
+          <t>4. Note any addenda, alternates, or special conditions</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="33" t="inlineStr">
+        <is>
+          <t>📖 See Manual: p. 4-7 — Getting Started &amp; Plan Orientation</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
         <is>
           <t>BLUEPRINT TAKEOFF WORKSHEET</t>
         </is>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>PROJECT INFORMATION</t>
         </is>
       </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>Project Name:</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Job Number:</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Builder/Customer:</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="n"/>
-      <c r="H22" s="43" t="inlineStr">
-        <is>
-          <t>Plan Orientation Diagram — See Manual p. 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Address:</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>Plan Set Date:</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>Revision Number:</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>Takeoff By:</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>Date Completed:</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Checked By:</t>
+          <t>Project Name:</t>
         </is>
       </c>
       <c r="B28" s="4" t="n"/>
     </row>
-    <row r="29"/>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Job Number:</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="n"/>
+    </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>BUILDING SPECIFICATIONS</t>
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Builder/Customer:</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="n"/>
+      <c r="H30" s="43" t="inlineStr">
+        <is>
+          <t>Plan Orientation Diagram — See Manual p. 5</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Building Type:</t>
+          <t>Address:</t>
         </is>
       </c>
       <c r="B31" s="4" t="n"/>
@@ -1395,7 +1572,7 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Stories:</t>
+          <t>Plan Set Date:</t>
         </is>
       </c>
       <c r="B32" s="4" t="n"/>
@@ -1403,7 +1580,7 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Foundation Type:</t>
+          <t>Revision Number:</t>
         </is>
       </c>
       <c r="B33" s="4" t="n"/>
@@ -1411,7 +1588,7 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Roof Type:</t>
+          <t>Takeoff By:</t>
         </is>
       </c>
       <c r="B34" s="4" t="n"/>
@@ -1419,7 +1596,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Total Square Footage:</t>
+          <t>Date Completed:</t>
         </is>
       </c>
       <c r="B35" s="4" t="n"/>
@@ -1427,7 +1604,7 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Wall Height:</t>
+          <t>Checked By:</t>
         </is>
       </c>
       <c r="B36" s="4" t="n"/>
@@ -1436,40 +1613,96 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
+          <t>BUILDING SPECIFICATIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Building Type:</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Stories:</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Foundation Type:</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Roof Type:</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Total Square Footage:</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Wall Height:</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="n"/>
+    </row>
+    <row r="45"/>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
           <t>REGIONAL NOTES (Southeast Texas)</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
+    <row r="47">
+      <c r="A47" t="inlineStr">
         <is>
           <t>• Slab foundations are standard (high water table)</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
+    <row r="48">
+      <c r="A48" t="inlineStr">
         <is>
           <t>• Consider humidity-resistant materials</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>• Windstorm requirements (hurricane zone)</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>• Treated lumber required for bottom plates</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr">
         <is>
           <t>• Additional anchor bolts per wind code</t>
         </is>
@@ -1500,7 +1733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M45"/>
+  <dimension ref="A1:M52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1654,498 +1887,566 @@
     </row>
     <row r="14"/>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="34" t="inlineStr">
+        <is>
+          <t>STEP 2 — WALL FRAMING TAKEOFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>INSTRUCTIONS:</t>
+        </is>
+      </c>
+      <c r="H16" s="35" t="inlineStr">
+        <is>
+          <t>💡 TIPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="27" t="inlineStr">
+        <is>
+          <t>1. Highlight all exterior walls on the floor plan</t>
+        </is>
+      </c>
+      <c r="H17" s="27" t="inlineStr">
+        <is>
+          <t>• Add extra studs for corners (3) and tees (2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="27" t="inlineStr">
+        <is>
+          <t>2. Label walls W1, W2, W3... moving clockwise from front left</t>
+        </is>
+      </c>
+      <c r="H18" s="27" t="inlineStr">
+        <is>
+          <t>• Use header schedule for kings/jacks—don't guess</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="27" t="inlineStr">
+        <is>
+          <t>3. Measure each wall and enter: length, height, stud spacing</t>
+        </is>
+      </c>
+      <c r="H19" s="27" t="inlineStr">
+        <is>
+          <t>• Remember the '+1' in stud count formula</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="27" t="inlineStr">
+        <is>
+          <t>4. Count corners, tees, and openings (windows/doors)</t>
+        </is>
+      </c>
+      <c r="H20" s="36" t="inlineStr">
+        <is>
+          <t>📖 Manual: p. 14-17 — Wall Framing</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>WALL FRAMING TAKEOFF</t>
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Wall ID</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>Length (ft)</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>Height (ft)</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr">
         <is>
           <t>Stud Spacing</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>Base Studs</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr">
         <is>
           <t>Corner Adds</t>
         </is>
       </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="H24" s="6" t="inlineStr">
         <is>
           <t>Opening Adj</t>
         </is>
       </c>
-      <c r="I17" s="6" t="inlineStr">
+      <c r="I24" s="6" t="inlineStr">
         <is>
           <t>Total Studs</t>
         </is>
       </c>
-      <c r="J17" s="6" t="inlineStr">
+      <c r="J24" s="6" t="inlineStr">
         <is>
           <t>Bottom Plate LF</t>
         </is>
       </c>
-      <c r="K17" s="6" t="inlineStr">
+      <c r="K24" s="6" t="inlineStr">
         <is>
           <t>Top Plate LF</t>
         </is>
       </c>
-      <c r="L17" s="6" t="inlineStr">
+      <c r="L24" s="6" t="inlineStr">
         <is>
           <t>Header Notes</t>
         </is>
       </c>
-      <c r="M17" s="6" t="inlineStr">
+      <c r="M24" s="6" t="inlineStr">
         <is>
           <t>Treated?</t>
         </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="F18">
-        <f>IF(C4="","",INT(C4*12/16)+1)</f>
-        <v/>
-      </c>
-      <c r="I18">
-        <f>IF(F4="","",F4+G4+H4)</f>
-        <v/>
-      </c>
-      <c r="J18">
-        <f>IF(C4="","",C4)</f>
-        <v/>
-      </c>
-      <c r="K18">
-        <f>IF(C4="","",C4*2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="F19">
-        <f>IF(C5="","",INT(C5*12/16)+1)</f>
-        <v/>
-      </c>
-      <c r="I19">
-        <f>IF(F5="","",F5+G5+H5)</f>
-        <v/>
-      </c>
-      <c r="J19">
-        <f>IF(C5="","",C5)</f>
-        <v/>
-      </c>
-      <c r="K19">
-        <f>IF(C5="","",C5*2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="F20">
-        <f>IF(C6="","",INT(C6*12/16)+1)</f>
-        <v/>
-      </c>
-      <c r="I20">
-        <f>IF(F6="","",F6+G6+H6)</f>
-        <v/>
-      </c>
-      <c r="J20">
-        <f>IF(C6="","",C6)</f>
-        <v/>
-      </c>
-      <c r="K20">
-        <f>IF(C6="","",C6*2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="F21">
-        <f>IF(C7="","",INT(C7*12/16)+1)</f>
-        <v/>
-      </c>
-      <c r="I21">
-        <f>IF(F7="","",F7+G7+H7)</f>
-        <v/>
-      </c>
-      <c r="J21">
-        <f>IF(C7="","",C7)</f>
-        <v/>
-      </c>
-      <c r="K21">
-        <f>IF(C7="","",C7*2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="F22">
-        <f>IF(C8="","",INT(C8*12/16)+1)</f>
-        <v/>
-      </c>
-      <c r="I22">
-        <f>IF(F8="","",F8+G8+H8)</f>
-        <v/>
-      </c>
-      <c r="J22">
-        <f>IF(C8="","",C8)</f>
-        <v/>
-      </c>
-      <c r="K22">
-        <f>IF(C8="","",C8*2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="F23">
-        <f>IF(C9="","",INT(C9*12/16)+1)</f>
-        <v/>
-      </c>
-      <c r="I23">
-        <f>IF(F9="","",F9+G9+H9)</f>
-        <v/>
-      </c>
-      <c r="J23">
-        <f>IF(C9="","",C9)</f>
-        <v/>
-      </c>
-      <c r="K23">
-        <f>IF(C9="","",C9*2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="F24">
-        <f>IF(C10="","",INT(C10*12/16)+1)</f>
-        <v/>
-      </c>
-      <c r="I24">
-        <f>IF(F10="","",F10+G10+H10)</f>
-        <v/>
-      </c>
-      <c r="J24">
-        <f>IF(C10="","",C10)</f>
-        <v/>
-      </c>
-      <c r="K24">
-        <f>IF(C10="","",C10*2)</f>
-        <v/>
       </c>
     </row>
     <row r="25">
       <c r="F25">
-        <f>IF(C11="","",INT(C11*12/16)+1)</f>
+        <f>IF(C4="","",INT(C4*12/16)+1)</f>
         <v/>
       </c>
       <c r="I25">
-        <f>IF(F11="","",F11+G11+H11)</f>
+        <f>IF(F4="","",F4+G4+H4)</f>
         <v/>
       </c>
       <c r="J25">
-        <f>IF(C11="","",C11)</f>
-        <v/>
-      </c>
-      <c r="K25" s="43" t="inlineStr">
-        <is>
-          <t>Wall Section — Manual p. 14-17</t>
-        </is>
+        <f>IF(C4="","",C4)</f>
+        <v/>
+      </c>
+      <c r="K25">
+        <f>IF(C4="","",C4*2)</f>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="F26">
-        <f>IF(C12="","",INT(C12*12/16)+1)</f>
+        <f>IF(C5="","",INT(C5*12/16)+1)</f>
         <v/>
       </c>
       <c r="I26">
-        <f>IF(F12="","",F12+G12+H12)</f>
+        <f>IF(F5="","",F5+G5+H5)</f>
         <v/>
       </c>
       <c r="J26">
-        <f>IF(C12="","",C12)</f>
+        <f>IF(C5="","",C5)</f>
         <v/>
       </c>
       <c r="K26">
-        <f>IF(C12="","",C12*2)</f>
+        <f>IF(C5="","",C5*2)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="F27">
-        <f>IF(C13="","",INT(C13*12/16)+1)</f>
+        <f>IF(C6="","",INT(C6*12/16)+1)</f>
         <v/>
       </c>
       <c r="I27">
-        <f>IF(F13="","",F13+G13+H13)</f>
+        <f>IF(F6="","",F6+G6+H6)</f>
         <v/>
       </c>
       <c r="J27">
-        <f>IF(C13="","",C13)</f>
+        <f>IF(C6="","",C6)</f>
         <v/>
       </c>
       <c r="K27">
-        <f>IF(C13="","",C13*2)</f>
+        <f>IF(C6="","",C6*2)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="F28">
-        <f>IF(C14="","",INT(C14*12/16)+1)</f>
+        <f>IF(C7="","",INT(C7*12/16)+1)</f>
         <v/>
       </c>
       <c r="I28">
-        <f>IF(F14="","",F14+G14+H14)</f>
+        <f>IF(F7="","",F7+G7+H7)</f>
         <v/>
       </c>
       <c r="J28">
-        <f>IF(C14="","",C14)</f>
+        <f>IF(C7="","",C7)</f>
         <v/>
       </c>
       <c r="K28">
-        <f>IF(C14="","",C14*2)</f>
+        <f>IF(C7="","",C7*2)</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="F29">
-        <f>IF(C15="","",INT(C15*12/16)+1)</f>
+        <f>IF(C8="","",INT(C8*12/16)+1)</f>
         <v/>
       </c>
       <c r="I29">
-        <f>IF(F15="","",F15+G15+H15)</f>
+        <f>IF(F8="","",F8+G8+H8)</f>
         <v/>
       </c>
       <c r="J29">
-        <f>IF(C15="","",C15)</f>
+        <f>IF(C8="","",C8)</f>
         <v/>
       </c>
       <c r="K29">
-        <f>IF(C15="","",C15*2)</f>
+        <f>IF(C8="","",C8*2)</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="F30">
-        <f>IF(C16="","",INT(C16*12/16)+1)</f>
+        <f>IF(C9="","",INT(C9*12/16)+1)</f>
         <v/>
       </c>
       <c r="I30">
-        <f>IF(F16="","",F16+G16+H16)</f>
+        <f>IF(F9="","",F9+G9+H9)</f>
         <v/>
       </c>
       <c r="J30">
-        <f>IF(C16="","",C16)</f>
+        <f>IF(C9="","",C9)</f>
         <v/>
       </c>
       <c r="K30">
-        <f>IF(C16="","",C16*2)</f>
+        <f>IF(C9="","",C9*2)</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="F31">
-        <f>IF(C17="","",INT(C17*12/16)+1)</f>
+        <f>IF(C10="","",INT(C10*12/16)+1)</f>
         <v/>
       </c>
       <c r="I31">
-        <f>IF(F17="","",F17+G17+H17)</f>
+        <f>IF(F10="","",F10+G10+H10)</f>
         <v/>
       </c>
       <c r="J31">
-        <f>IF(C17="","",C17)</f>
+        <f>IF(C10="","",C10)</f>
         <v/>
       </c>
       <c r="K31">
-        <f>IF(C17="","",C17*2)</f>
+        <f>IF(C10="","",C10*2)</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="F32">
-        <f>IF(C18="","",INT(C18*12/16)+1)</f>
+        <f>IF(C11="","",INT(C11*12/16)+1)</f>
         <v/>
       </c>
       <c r="I32">
-        <f>IF(F18="","",F18+G18+H18)</f>
+        <f>IF(F11="","",F11+G11+H11)</f>
         <v/>
       </c>
       <c r="J32">
-        <f>IF(C18="","",C18)</f>
-        <v/>
-      </c>
-      <c r="K32">
-        <f>IF(C18="","",C18*2)</f>
-        <v/>
+        <f>IF(C11="","",C11)</f>
+        <v/>
+      </c>
+      <c r="K32" s="43" t="inlineStr">
+        <is>
+          <t>Wall Section — Manual p. 14-17</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="F33">
-        <f>IF(C19="","",INT(C19*12/16)+1)</f>
+        <f>IF(C12="","",INT(C12*12/16)+1)</f>
         <v/>
       </c>
       <c r="I33">
-        <f>IF(F19="","",F19+G19+H19)</f>
+        <f>IF(F12="","",F12+G12+H12)</f>
         <v/>
       </c>
       <c r="J33">
-        <f>IF(C19="","",C19)</f>
+        <f>IF(C12="","",C12)</f>
         <v/>
       </c>
       <c r="K33">
-        <f>IF(C19="","",C19*2)</f>
+        <f>IF(C12="","",C12*2)</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="F34">
-        <f>IF(C20="","",INT(C20*12/16)+1)</f>
+        <f>IF(C13="","",INT(C13*12/16)+1)</f>
         <v/>
       </c>
       <c r="I34">
-        <f>IF(F20="","",F20+G20+H20)</f>
+        <f>IF(F13="","",F13+G13+H13)</f>
         <v/>
       </c>
       <c r="J34">
-        <f>IF(C20="","",C20)</f>
+        <f>IF(C13="","",C13)</f>
         <v/>
       </c>
       <c r="K34">
-        <f>IF(C20="","",C20*2)</f>
+        <f>IF(C13="","",C13*2)</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="F35">
-        <f>IF(C21="","",INT(C21*12/16)+1)</f>
+        <f>IF(C14="","",INT(C14*12/16)+1)</f>
         <v/>
       </c>
       <c r="I35">
-        <f>IF(F21="","",F21+G21+H21)</f>
+        <f>IF(F14="","",F14+G14+H14)</f>
         <v/>
       </c>
       <c r="J35">
-        <f>IF(C21="","",C21)</f>
+        <f>IF(C14="","",C14)</f>
         <v/>
       </c>
       <c r="K35">
-        <f>IF(C21="","",C21*2)</f>
+        <f>IF(C14="","",C14*2)</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="F36">
-        <f>IF(C22="","",INT(C22*12/16)+1)</f>
+        <f>IF(C15="","",INT(C15*12/16)+1)</f>
         <v/>
       </c>
       <c r="I36">
-        <f>IF(F22="","",F22+G22+H22)</f>
+        <f>IF(F15="","",F15+G15+H15)</f>
         <v/>
       </c>
       <c r="J36">
-        <f>IF(C22="","",C22)</f>
+        <f>IF(C15="","",C15)</f>
         <v/>
       </c>
       <c r="K36">
-        <f>IF(C22="","",C22*2)</f>
+        <f>IF(C15="","",C15*2)</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="F37">
+        <f>IF(C16="","",INT(C16*12/16)+1)</f>
+        <v/>
+      </c>
+      <c r="I37">
+        <f>IF(F16="","",F16+G16+H16)</f>
+        <v/>
+      </c>
+      <c r="J37">
+        <f>IF(C16="","",C16)</f>
+        <v/>
+      </c>
+      <c r="K37">
+        <f>IF(C16="","",C16*2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="F38">
+        <f>IF(C17="","",INT(C17*12/16)+1)</f>
+        <v/>
+      </c>
+      <c r="I38">
+        <f>IF(F17="","",F17+G17+H17)</f>
+        <v/>
+      </c>
+      <c r="J38">
+        <f>IF(C17="","",C17)</f>
+        <v/>
+      </c>
+      <c r="K38">
+        <f>IF(C17="","",C17*2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="F39">
+        <f>IF(C18="","",INT(C18*12/16)+1)</f>
+        <v/>
+      </c>
+      <c r="I39">
+        <f>IF(F18="","",F18+G18+H18)</f>
+        <v/>
+      </c>
+      <c r="J39">
+        <f>IF(C18="","",C18)</f>
+        <v/>
+      </c>
+      <c r="K39">
+        <f>IF(C18="","",C18*2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="F40">
+        <f>IF(C19="","",INT(C19*12/16)+1)</f>
+        <v/>
+      </c>
+      <c r="I40">
+        <f>IF(F19="","",F19+G19+H19)</f>
+        <v/>
+      </c>
+      <c r="J40">
+        <f>IF(C19="","",C19)</f>
+        <v/>
+      </c>
+      <c r="K40">
+        <f>IF(C19="","",C19*2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="F41">
+        <f>IF(C20="","",INT(C20*12/16)+1)</f>
+        <v/>
+      </c>
+      <c r="I41">
+        <f>IF(F20="","",F20+G20+H20)</f>
+        <v/>
+      </c>
+      <c r="J41">
+        <f>IF(C20="","",C20)</f>
+        <v/>
+      </c>
+      <c r="K41">
+        <f>IF(C20="","",C20*2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="F42">
+        <f>IF(C21="","",INT(C21*12/16)+1)</f>
+        <v/>
+      </c>
+      <c r="I42">
+        <f>IF(F21="","",F21+G21+H21)</f>
+        <v/>
+      </c>
+      <c r="J42">
+        <f>IF(C21="","",C21)</f>
+        <v/>
+      </c>
+      <c r="K42">
+        <f>IF(C21="","",C21*2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="F43">
+        <f>IF(C22="","",INT(C22*12/16)+1)</f>
+        <v/>
+      </c>
+      <c r="I43">
+        <f>IF(F22="","",F22+G22+H22)</f>
+        <v/>
+      </c>
+      <c r="J43">
+        <f>IF(C22="","",C22)</f>
+        <v/>
+      </c>
+      <c r="K43">
+        <f>IF(C22="","",C22*2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="F44">
         <f>IF(C23="","",INT(C23*12/16)+1)</f>
         <v/>
       </c>
-      <c r="I37">
+      <c r="I44">
         <f>IF(F23="","",F23+G23+H23)</f>
         <v/>
       </c>
-      <c r="J37">
+      <c r="J44">
         <f>IF(C23="","",C23)</f>
         <v/>
       </c>
-      <c r="K37">
+      <c r="K44">
         <f>IF(C23="","",C23*2)</f>
         <v/>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="I38" s="7">
+      <c r="I45" s="7">
         <f>SUM(I4:I23)</f>
         <v/>
       </c>
-      <c r="J38" s="7">
+      <c r="J45" s="7">
         <f>SUM(J4:J23)</f>
         <v/>
       </c>
-      <c r="K38" s="7">
+      <c r="K45" s="7">
         <f>SUM(K4:K23)</f>
         <v/>
       </c>
     </row>
-    <row r="39"/>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+    <row r="46"/>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>INSTRUCTIONS:</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
+    <row r="48">
+      <c r="A48" t="inlineStr">
         <is>
           <t>1. Enter wall length in feet (e.g., 24)</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>2. Enter wall height in feet (e.g., 8)</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>3. Stud spacing: 16 or 24 (16 is most common)</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr">
         <is>
           <t>4. Corner Adds: +2 for exterior corners, +1 for T-intersections</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
+    <row r="52">
+      <c r="A52" t="inlineStr">
         <is>
           <t>5. Opening Adj: Count king/jack studs minus displaced studs</t>
         </is>
@@ -2176,7 +2477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N36"/>
+  <dimension ref="A1:N43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2330,432 +2631,500 @@
     </row>
     <row r="14"/>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="37" t="inlineStr">
+        <is>
+          <t>STEP 3 — ROOF TAKEOFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>INSTRUCTIONS:</t>
+        </is>
+      </c>
+      <c r="H16" s="35" t="inlineStr">
+        <is>
+          <t>💡 TIPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="27" t="inlineStr">
+        <is>
+          <t>1. Locate roof plan and framing details</t>
+        </is>
+      </c>
+      <c r="H17" s="27" t="inlineStr">
+        <is>
+          <t>• Include overhangs in width/length for sheathing</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="27" t="inlineStr">
+        <is>
+          <t>2. For each roof plane, record: width, length, pitch, overhang</t>
+        </is>
+      </c>
+      <c r="H18" s="27" t="inlineStr">
+        <is>
+          <t>• Don't forget porch and garage roofs</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="27" t="inlineStr">
+        <is>
+          <t>3. Use slope factor table to calculate sheathing area</t>
+        </is>
+      </c>
+      <c r="H19" s="27" t="inlineStr">
+        <is>
+          <t>• Add 10-15% waste for shingles</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="27" t="inlineStr">
+        <is>
+          <t>4. Remember: porch and garage roofs count too!</t>
+        </is>
+      </c>
+      <c r="H20" s="36" t="inlineStr">
+        <is>
+          <t>📖 Manual: p. 18-20 — Roof Takeoff</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>ROOF TAKEOFF CALCULATOR</t>
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>SLOPE FACTORS (Reference)</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>ROOF PLANE CALCULATIONS</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>Pitch</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Factor</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D25" s="9" t="inlineStr">
         <is>
           <t>Plane ID</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E25" s="9" t="inlineStr">
         <is>
           <t>Length (ft)</t>
         </is>
       </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="F25" s="9" t="inlineStr">
         <is>
           <t>Width (ft)</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
+      <c r="G25" s="9" t="inlineStr">
         <is>
           <t>Pitch</t>
         </is>
       </c>
-      <c r="H18" s="9" t="inlineStr">
+      <c r="H25" s="9" t="inlineStr">
         <is>
           <t>Slope Factor</t>
         </is>
       </c>
-      <c r="I18" s="9" t="inlineStr">
+      <c r="I25" s="9" t="inlineStr">
         <is>
           <t>Horiz Area (SF)</t>
         </is>
       </c>
-      <c r="J18" s="9" t="inlineStr">
+      <c r="J25" s="9" t="inlineStr">
         <is>
           <t>Surface Area (SF)</t>
         </is>
       </c>
-      <c r="K18" s="9" t="inlineStr">
+      <c r="K25" s="9" t="inlineStr">
         <is>
           <t>Sheathing Sheets</t>
         </is>
       </c>
-      <c r="L18" s="9" t="inlineStr">
+      <c r="L25" s="9" t="inlineStr">
         <is>
           <t>Waste %</t>
         </is>
       </c>
-      <c r="M18" s="9" t="inlineStr">
+      <c r="M25" s="9" t="inlineStr">
         <is>
           <t>Total Sheets</t>
         </is>
       </c>
-      <c r="N18" s="9" t="inlineStr">
+      <c r="N25" s="9" t="inlineStr">
         <is>
           <t>Bundles</t>
         </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>4:12</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>1.054</v>
-      </c>
-      <c r="I19">
-        <f>IF(E5="","",E5*F5)</f>
-        <v/>
-      </c>
-      <c r="J19">
-        <f>IF(I5="","",I5*H5)</f>
-        <v/>
-      </c>
-      <c r="K19">
-        <f>IF(J5="","",J5/32)</f>
-        <v/>
-      </c>
-      <c r="M19">
-        <f>IF(K5="","",ROUNDUP(K5*(1+L5/100),0))</f>
-        <v/>
-      </c>
-      <c r="N19">
-        <f>IF(J5="","",ROUNDUP(J5/100*3,0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>5:12</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>1.083</v>
-      </c>
-      <c r="I20">
-        <f>IF(E6="","",E6*F6)</f>
-        <v/>
-      </c>
-      <c r="J20">
-        <f>IF(I6="","",I6*H6)</f>
-        <v/>
-      </c>
-      <c r="K20">
-        <f>IF(J6="","",J6/32)</f>
-        <v/>
-      </c>
-      <c r="M20">
-        <f>IF(K6="","",ROUNDUP(K6*(1+L6/100),0))</f>
-        <v/>
-      </c>
-      <c r="N20">
-        <f>IF(J6="","",ROUNDUP(J6/100*3,0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>6:12</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>1.118</v>
-      </c>
-      <c r="I21">
-        <f>IF(E7="","",E7*F7)</f>
-        <v/>
-      </c>
-      <c r="J21">
-        <f>IF(I7="","",I7*H7)</f>
-        <v/>
-      </c>
-      <c r="K21">
-        <f>IF(J7="","",J7/32)</f>
-        <v/>
-      </c>
-      <c r="M21">
-        <f>IF(K7="","",ROUNDUP(K7*(1+L7/100),0))</f>
-        <v/>
-      </c>
-      <c r="N21">
-        <f>IF(J7="","",ROUNDUP(J7/100*3,0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>7:12</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>1.158</v>
-      </c>
-      <c r="I22">
-        <f>IF(E8="","",E8*F8)</f>
-        <v/>
-      </c>
-      <c r="J22">
-        <f>IF(I8="","",I8*H8)</f>
-        <v/>
-      </c>
-      <c r="K22" s="43" t="inlineStr">
-        <is>
-          <t>Roof Plan &amp; Pitch — Manual p. 18-20</t>
-        </is>
-      </c>
-      <c r="M22">
-        <f>IF(K8="","",ROUNDUP(K8*(1+L8/100),0))</f>
-        <v/>
-      </c>
-      <c r="N22">
-        <f>IF(J8="","",ROUNDUP(J8/100*3,0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>8:12</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>1.202</v>
-      </c>
-      <c r="I23">
-        <f>IF(E9="","",E9*F9)</f>
-        <v/>
-      </c>
-      <c r="J23">
-        <f>IF(I9="","",I9*H9)</f>
-        <v/>
-      </c>
-      <c r="K23">
-        <f>IF(J9="","",J9/32)</f>
-        <v/>
-      </c>
-      <c r="M23">
-        <f>IF(K9="","",ROUNDUP(K9*(1+L9/100),0))</f>
-        <v/>
-      </c>
-      <c r="N23">
-        <f>IF(J9="","",ROUNDUP(J9/100*3,0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>9:12</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="I24">
-        <f>IF(E10="","",E10*F10)</f>
-        <v/>
-      </c>
-      <c r="J24">
-        <f>IF(I10="","",I10*H10)</f>
-        <v/>
-      </c>
-      <c r="K24">
-        <f>IF(J10="","",J10/32)</f>
-        <v/>
-      </c>
-      <c r="M24">
-        <f>IF(K10="","",ROUNDUP(K10*(1+L10/100),0))</f>
-        <v/>
-      </c>
-      <c r="N24">
-        <f>IF(J10="","",ROUNDUP(J10/100*3,0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>10:12</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>1.302</v>
-      </c>
-      <c r="I25">
-        <f>IF(E11="","",E11*F11)</f>
-        <v/>
-      </c>
-      <c r="J25">
-        <f>IF(I11="","",I11*H11)</f>
-        <v/>
-      </c>
-      <c r="K25">
-        <f>IF(J11="","",J11/32)</f>
-        <v/>
-      </c>
-      <c r="M25">
-        <f>IF(K11="","",ROUNDUP(K11*(1+L11/100),0))</f>
-        <v/>
-      </c>
-      <c r="N25">
-        <f>IF(J11="","",ROUNDUP(J11/100*3,0))</f>
-        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>4:12</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1.054</v>
+      </c>
+      <c r="I26">
+        <f>IF(E5="","",E5*F5)</f>
+        <v/>
+      </c>
+      <c r="J26">
+        <f>IF(I5="","",I5*H5)</f>
+        <v/>
+      </c>
+      <c r="K26">
+        <f>IF(J5="","",J5/32)</f>
+        <v/>
+      </c>
+      <c r="M26">
+        <f>IF(K5="","",ROUNDUP(K5*(1+L5/100),0))</f>
+        <v/>
+      </c>
+      <c r="N26">
+        <f>IF(J5="","",ROUNDUP(J5/100*3,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>5:12</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1.083</v>
+      </c>
+      <c r="I27">
+        <f>IF(E6="","",E6*F6)</f>
+        <v/>
+      </c>
+      <c r="J27">
+        <f>IF(I6="","",I6*H6)</f>
+        <v/>
+      </c>
+      <c r="K27">
+        <f>IF(J6="","",J6/32)</f>
+        <v/>
+      </c>
+      <c r="M27">
+        <f>IF(K6="","",ROUNDUP(K6*(1+L6/100),0))</f>
+        <v/>
+      </c>
+      <c r="N27">
+        <f>IF(J6="","",ROUNDUP(J6/100*3,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>6:12</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1.118</v>
+      </c>
+      <c r="I28">
+        <f>IF(E7="","",E7*F7)</f>
+        <v/>
+      </c>
+      <c r="J28">
+        <f>IF(I7="","",I7*H7)</f>
+        <v/>
+      </c>
+      <c r="K28">
+        <f>IF(J7="","",J7/32)</f>
+        <v/>
+      </c>
+      <c r="M28">
+        <f>IF(K7="","",ROUNDUP(K7*(1+L7/100),0))</f>
+        <v/>
+      </c>
+      <c r="N28">
+        <f>IF(J7="","",ROUNDUP(J7/100*3,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>7:12</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1.158</v>
+      </c>
+      <c r="I29">
+        <f>IF(E8="","",E8*F8)</f>
+        <v/>
+      </c>
+      <c r="J29">
+        <f>IF(I8="","",I8*H8)</f>
+        <v/>
+      </c>
+      <c r="K29" s="43" t="inlineStr">
+        <is>
+          <t>Roof Plan &amp; Pitch — Manual p. 18-20</t>
+        </is>
+      </c>
+      <c r="M29">
+        <f>IF(K8="","",ROUNDUP(K8*(1+L8/100),0))</f>
+        <v/>
+      </c>
+      <c r="N29">
+        <f>IF(J8="","",ROUNDUP(J8/100*3,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>8:12</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1.202</v>
+      </c>
+      <c r="I30">
+        <f>IF(E9="","",E9*F9)</f>
+        <v/>
+      </c>
+      <c r="J30">
+        <f>IF(I9="","",I9*H9)</f>
+        <v/>
+      </c>
+      <c r="K30">
+        <f>IF(J9="","",J9/32)</f>
+        <v/>
+      </c>
+      <c r="M30">
+        <f>IF(K9="","",ROUNDUP(K9*(1+L9/100),0))</f>
+        <v/>
+      </c>
+      <c r="N30">
+        <f>IF(J9="","",ROUNDUP(J9/100*3,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>9:12</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="I31">
+        <f>IF(E10="","",E10*F10)</f>
+        <v/>
+      </c>
+      <c r="J31">
+        <f>IF(I10="","",I10*H10)</f>
+        <v/>
+      </c>
+      <c r="K31">
+        <f>IF(J10="","",J10/32)</f>
+        <v/>
+      </c>
+      <c r="M31">
+        <f>IF(K10="","",ROUNDUP(K10*(1+L10/100),0))</f>
+        <v/>
+      </c>
+      <c r="N31">
+        <f>IF(J10="","",ROUNDUP(J10/100*3,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>10:12</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1.302</v>
+      </c>
+      <c r="I32">
+        <f>IF(E11="","",E11*F11)</f>
+        <v/>
+      </c>
+      <c r="J32">
+        <f>IF(I11="","",I11*H11)</f>
+        <v/>
+      </c>
+      <c r="K32">
+        <f>IF(J11="","",J11/32)</f>
+        <v/>
+      </c>
+      <c r="M32">
+        <f>IF(K11="","",ROUNDUP(K11*(1+L11/100),0))</f>
+        <v/>
+      </c>
+      <c r="N32">
+        <f>IF(J11="","",ROUNDUP(J11/100*3,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>12:12</t>
         </is>
       </c>
-      <c r="B26" t="n">
+      <c r="B33" t="n">
         <v>1.414</v>
       </c>
-      <c r="I26">
+      <c r="I33">
         <f>IF(E12="","",E12*F12)</f>
         <v/>
       </c>
-      <c r="J26">
+      <c r="J33">
         <f>IF(I12="","",I12*H12)</f>
         <v/>
       </c>
-      <c r="K26">
+      <c r="K33">
         <f>IF(J12="","",J12/32)</f>
         <v/>
       </c>
-      <c r="M26">
+      <c r="M33">
         <f>IF(K12="","",ROUNDUP(K12*(1+L12/100),0))</f>
         <v/>
       </c>
-      <c r="N26">
+      <c r="N33">
         <f>IF(J12="","",ROUNDUP(J12/100*3,0))</f>
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="I27">
+    <row r="34">
+      <c r="I34">
         <f>IF(E13="","",E13*F13)</f>
         <v/>
       </c>
-      <c r="J27">
+      <c r="J34">
         <f>IF(I13="","",I13*H13)</f>
         <v/>
       </c>
-      <c r="K27">
+      <c r="K34">
         <f>IF(J13="","",J13/32)</f>
         <v/>
       </c>
-      <c r="M27">
+      <c r="M34">
         <f>IF(K13="","",ROUNDUP(K13*(1+L13/100),0))</f>
         <v/>
       </c>
-      <c r="N27">
+      <c r="N34">
         <f>IF(J13="","",ROUNDUP(J13/100*3,0))</f>
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="I28">
+    <row r="35">
+      <c r="I35">
         <f>IF(E14="","",E14*F14)</f>
         <v/>
       </c>
-      <c r="J28">
+      <c r="J35">
         <f>IF(I14="","",I14*H14)</f>
         <v/>
       </c>
-      <c r="K28">
+      <c r="K35">
         <f>IF(J14="","",J14/32)</f>
         <v/>
       </c>
-      <c r="M28">
+      <c r="M35">
         <f>IF(K14="","",ROUNDUP(K14*(1+L14/100),0))</f>
         <v/>
       </c>
-      <c r="N28">
+      <c r="N35">
         <f>IF(J14="","",ROUNDUP(J14/100*3,0))</f>
         <v/>
       </c>
     </row>
-    <row r="29"/>
-    <row r="30">
-      <c r="D30" s="3" t="inlineStr">
+    <row r="36"/>
+    <row r="37">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="J30" s="7">
+      <c r="J37" s="7">
         <f>SUM(J5:J15)</f>
         <v/>
       </c>
-      <c r="K30" s="7">
+      <c r="K37" s="7">
         <f>SUM(K5:K15)</f>
         <v/>
       </c>
-      <c r="M30" s="7">
+      <c r="M37" s="7">
         <f>SUM(M5:M15)</f>
         <v/>
       </c>
-      <c r="N30" s="7">
+      <c r="N37" s="7">
         <f>SUM(N5:N15)</f>
         <v/>
       </c>
     </row>
-    <row r="31"/>
-    <row r="32">
-      <c r="D32" s="8" t="inlineStr">
+    <row r="38"/>
+    <row r="39">
+      <c r="D39" s="8" t="inlineStr">
         <is>
           <t>NOTES:</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="D33" t="inlineStr">
+    <row r="40">
+      <c r="D40" t="inlineStr">
         <is>
           <t>• One 4x8 sheet = 32 square feet</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="D34" t="inlineStr">
+    <row r="41">
+      <c r="D41" t="inlineStr">
         <is>
           <t>• Typical waste factor: 10-15% for cuts and starter</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="D35" t="inlineStr">
+    <row r="42">
+      <c r="D42" t="inlineStr">
         <is>
           <t>• Shingles: 3 bundles = 1 square (100 SF)</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="D36" t="inlineStr">
+    <row r="43">
+      <c r="D43" t="inlineStr">
         <is>
           <t>• Hip and ridge cap: Add 10% to total bundles</t>
         </is>
@@ -2787,7 +3156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2936,288 +3305,356 @@
     </row>
     <row r="14"/>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="38" t="inlineStr">
+        <is>
+          <t>STEP 1 — FOUNDATION &amp; SLAB TAKEOFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>INSTRUCTIONS:</t>
+        </is>
+      </c>
+      <c r="F16" s="35" t="inlineStr">
+        <is>
+          <t>💡 TIPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="31" t="inlineStr">
+        <is>
+          <t>1. Locate foundation/structural sheets in the plan set</t>
+        </is>
+      </c>
+      <c r="F17" s="27" t="inlineStr">
+        <is>
+          <t>• Include porches and garage slabs</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="31" t="inlineStr">
+        <is>
+          <t>2. Trace the perimeter of the slab and any interior beams</t>
+        </is>
+      </c>
+      <c r="F18" s="27" t="inlineStr">
+        <is>
+          <t>• Note any assumed beam sizes for review</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="31" t="inlineStr">
+        <is>
+          <t>3. Measure each segment and enter lengths in the table below</t>
+        </is>
+      </c>
+      <c r="F19" s="27" t="inlineStr">
+        <is>
+          <t>• Remember to convert thickness to feet</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="31" t="inlineStr">
+        <is>
+          <t>4. Record slab thickness, beam sizes, and notes/assumptions</t>
+        </is>
+      </c>
+      <c r="F20" s="36" t="inlineStr">
+        <is>
+          <t>📖 Manual: p. 8-10 — Foundation</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>FOUNDATION &amp; CONCRETE TAKEOFF</t>
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>SLAB CALCULATIONS</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>Element</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>Length (ft)</t>
         </is>
       </c>
-      <c r="C18" s="10" t="inlineStr">
+      <c r="C25" s="10" t="inlineStr">
         <is>
           <t>Width (ft)</t>
         </is>
       </c>
-      <c r="D18" s="10" t="inlineStr">
+      <c r="D25" s="10" t="inlineStr">
         <is>
           <t>Thickness (in)</t>
         </is>
       </c>
-      <c r="E18" s="10" t="inlineStr">
+      <c r="E25" s="10" t="inlineStr">
         <is>
           <t>Cu Ft</t>
         </is>
       </c>
-      <c r="F18" s="10" t="inlineStr">
+      <c r="F25" s="10" t="inlineStr">
         <is>
           <t>Cu Yd</t>
         </is>
       </c>
-      <c r="G18" s="10" t="inlineStr">
+      <c r="G25" s="10" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="E19">
+    <row r="26">
+      <c r="E26">
         <f>IF(B5="","",B5*C5*(D5/12))</f>
         <v/>
       </c>
-      <c r="F19">
+      <c r="F26">
         <f>IF(E5="","",E5/27)</f>
         <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="E20">
-        <f>IF(B6="","",B6*C6*(D6/12))</f>
-        <v/>
-      </c>
-      <c r="F20">
-        <f>IF(E6="","",E6/27)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="E21">
-        <f>IF(B7="","",B7*C7*(D7/12))</f>
-        <v/>
-      </c>
-      <c r="F21">
-        <f>IF(E7="","",E7/27)</f>
-        <v/>
-      </c>
-      <c r="J21" s="43" t="inlineStr">
-        <is>
-          <t>Foundation Section — Manual p. 8-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="E22">
-        <f>IF(B8="","",B8*C8*(D8/12))</f>
-        <v/>
-      </c>
-      <c r="F22">
-        <f>IF(E8="","",E8/27)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="E23">
-        <f>IF(B9="","",B9*C9*(D9/12))</f>
-        <v/>
-      </c>
-      <c r="F23">
-        <f>IF(E9="","",E9/27)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24"/>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>PERIMETER FOOTING</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="B26" s="10" t="inlineStr">
-        <is>
-          <t>Length (ft)</t>
-        </is>
-      </c>
-      <c r="C26" s="10" t="inlineStr">
-        <is>
-          <t>Width (in)</t>
-        </is>
-      </c>
-      <c r="D26" s="10" t="inlineStr">
-        <is>
-          <t>Depth (in)</t>
-        </is>
-      </c>
-      <c r="E26" s="10" t="inlineStr">
-        <is>
-          <t>Cu Ft</t>
-        </is>
-      </c>
-      <c r="F26" s="10" t="inlineStr">
-        <is>
-          <t>Cu Yd</t>
-        </is>
-      </c>
-      <c r="G26" s="10" t="inlineStr">
-        <is>
-          <t>Rebar LF</t>
-        </is>
       </c>
     </row>
     <row r="27">
       <c r="E27">
-        <f>IF(B13="","",B13*(C13/12)*(D13/12))</f>
+        <f>IF(B6="","",B6*C6*(D6/12))</f>
         <v/>
       </c>
       <c r="F27">
-        <f>IF(E13="","",E13/27)</f>
-        <v/>
-      </c>
-      <c r="G27">
-        <f>IF(B13="","",B13*2)</f>
+        <f>IF(E6="","",E6/27)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="E28">
-        <f>IF(B14="","",B14*(C14/12)*(D14/12))</f>
+        <f>IF(B7="","",B7*C7*(D7/12))</f>
         <v/>
       </c>
       <c r="F28">
-        <f>IF(E14="","",E14/27)</f>
-        <v/>
-      </c>
-      <c r="G28">
-        <f>IF(B14="","",B14*2)</f>
-        <v/>
+        <f>IF(E7="","",E7/27)</f>
+        <v/>
+      </c>
+      <c r="J28" s="43" t="inlineStr">
+        <is>
+          <t>Foundation Section — Manual p. 8-10</t>
+        </is>
       </c>
     </row>
     <row r="29">
       <c r="E29">
-        <f>IF(B15="","",B15*(C15/12)*(D15/12))</f>
+        <f>IF(B8="","",B8*C8*(D8/12))</f>
         <v/>
       </c>
       <c r="F29">
-        <f>IF(E15="","",E15/27)</f>
-        <v/>
-      </c>
-      <c r="G29">
-        <f>IF(B15="","",B15*2)</f>
+        <f>IF(E8="","",E8/27)</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="E30">
+        <f>IF(B9="","",B9*C9*(D9/12))</f>
+        <v/>
+      </c>
+      <c r="F30">
+        <f>IF(E9="","",E9/27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>PERIMETER FOOTING</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>Length (ft)</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>Width (in)</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>Depth (in)</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>Cu Ft</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>Cu Yd</t>
+        </is>
+      </c>
+      <c r="G33" s="10" t="inlineStr">
+        <is>
+          <t>Rebar LF</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="E34">
+        <f>IF(B13="","",B13*(C13/12)*(D13/12))</f>
+        <v/>
+      </c>
+      <c r="F34">
+        <f>IF(E13="","",E13/27)</f>
+        <v/>
+      </c>
+      <c r="G34">
+        <f>IF(B13="","",B13*2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="E35">
+        <f>IF(B14="","",B14*(C14/12)*(D14/12))</f>
+        <v/>
+      </c>
+      <c r="F35">
+        <f>IF(E14="","",E14/27)</f>
+        <v/>
+      </c>
+      <c r="G35">
+        <f>IF(B14="","",B14*2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="E36">
+        <f>IF(B15="","",B15*(C15/12)*(D15/12))</f>
+        <v/>
+      </c>
+      <c r="F36">
+        <f>IF(E15="","",E15/27)</f>
+        <v/>
+      </c>
+      <c r="G36">
+        <f>IF(B15="","",B15*2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="E37">
         <f>IF(B16="","",B16*(C16/12)*(D16/12))</f>
         <v/>
       </c>
-      <c r="F30">
+      <c r="F37">
         <f>IF(E16="","",E16/27)</f>
         <v/>
       </c>
-      <c r="G30">
+      <c r="G37">
         <f>IF(B16="","",B16*2)</f>
         <v/>
       </c>
     </row>
-    <row r="31">
-      <c r="E31">
+    <row r="38">
+      <c r="E38">
         <f>IF(B17="","",B17*(C17/12)*(D17/12))</f>
         <v/>
       </c>
-      <c r="F31">
+      <c r="F38">
         <f>IF(E17="","",E17/27)</f>
         <v/>
       </c>
-      <c r="G31">
+      <c r="G38">
         <f>IF(B17="","",B17*2)</f>
         <v/>
       </c>
     </row>
-    <row r="32"/>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+    <row r="39"/>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>TOTAL CONCRETE</t>
         </is>
       </c>
-      <c r="F33" s="7">
+      <c r="F40" s="7">
         <f>SUM(F5:F9,F13:F18)</f>
         <v/>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>TOTAL REBAR</t>
         </is>
       </c>
-      <c r="G34" s="7">
+      <c r="G41" s="7">
         <f>SUM(G13:G18)</f>
         <v/>
       </c>
     </row>
-    <row r="35"/>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+    <row r="42"/>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>CONVERSION FACTORS:</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t>• 1 cubic yard = 27 cubic feet</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
+    <row r="45">
+      <c r="A45" t="inlineStr">
         <is>
           <t>• Add 5-10% waste for concrete</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t>• Standard slab thickness: 4 inches</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
+    <row r="47">
+      <c r="A47" t="inlineStr">
         <is>
           <t>• Perimeter footing: typically 16" wide x 12" deep minimum</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
+    <row r="48">
+      <c r="A48" t="inlineStr">
         <is>
           <t>• Southeast Texas: All bottom plates must be treated lumber</t>
         </is>
@@ -3248,7 +3685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3400,405 +3837,473 @@
     </row>
     <row r="14"/>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="39" t="inlineStr">
+        <is>
+          <t>STEP 4 — SIDING, SOFFIT, FASCIA &amp; EXTERIOR TRIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>INSTRUCTIONS:</t>
+        </is>
+      </c>
+      <c r="G16" s="35" t="inlineStr">
+        <is>
+          <t>💡 TIPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="27" t="inlineStr">
+        <is>
+          <t>1. Use each elevation (Front, Rear, Left, Right)</t>
+        </is>
+      </c>
+      <c r="G17" s="27" t="inlineStr">
+        <is>
+          <t>• Add 10% waste for siding</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="27" t="inlineStr">
+        <is>
+          <t>2. Measure wall width, height, and gable rise if applicable</t>
+        </is>
+      </c>
+      <c r="G18" s="27" t="inlineStr">
+        <is>
+          <t>• Don't subtract small openings &lt; 10 SF</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="27" t="inlineStr">
+        <is>
+          <t>3. Subtract windows/doors based on siding type</t>
+        </is>
+      </c>
+      <c r="G19" s="27" t="inlineStr">
+        <is>
+          <t>• Measure trim/fascia separately for each edge</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="27" t="inlineStr">
+        <is>
+          <t>4. Calculate linear feet for trim, fascia, soffit</t>
+        </is>
+      </c>
+      <c r="G20" s="36" t="inlineStr">
+        <is>
+          <t>📖 Manual: p. 21-23 — Siding</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>SIDING &amp; EXTERIOR MATERIALS TAKEOFF</t>
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>Elevation</t>
         </is>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>LF</t>
         </is>
       </c>
-      <c r="C17" s="11" t="inlineStr">
+      <c r="C24" s="11" t="inlineStr">
         <is>
           <t>Plate Ht (ft)</t>
         </is>
       </c>
-      <c r="D17" s="11" t="inlineStr">
+      <c r="D24" s="11" t="inlineStr">
         <is>
           <t>Gable Rise (ft)</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>Wall Area</t>
         </is>
       </c>
-      <c r="F17" s="11" t="inlineStr">
+      <c r="F24" s="11" t="inlineStr">
         <is>
           <t>Gable Area</t>
         </is>
       </c>
-      <c r="G17" s="11" t="inlineStr">
+      <c r="G24" s="11" t="inlineStr">
         <is>
           <t>Gross SF</t>
         </is>
       </c>
-      <c r="H17" s="11" t="inlineStr">
+      <c r="H24" s="11" t="inlineStr">
         <is>
           <t>Openings SF</t>
         </is>
       </c>
-      <c r="I17" s="11" t="inlineStr">
+      <c r="I24" s="11" t="inlineStr">
         <is>
           <t>Net SF</t>
         </is>
       </c>
-      <c r="J17" s="11" t="inlineStr">
+      <c r="J24" s="11" t="inlineStr">
         <is>
           <t>Waste %</t>
         </is>
       </c>
-      <c r="K17" s="11" t="inlineStr">
+      <c r="K24" s="11" t="inlineStr">
         <is>
           <t>Order SF</t>
         </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="E18">
-        <f>IF(B4="","",B4*C4)</f>
-        <v/>
-      </c>
-      <c r="F18">
-        <f>IF(D4="","",B4*D4/2)</f>
-        <v/>
-      </c>
-      <c r="G18">
-        <f>IF(E4="","",E4+F4)</f>
-        <v/>
-      </c>
-      <c r="I18">
-        <f>IF(G4="","",G4-H4)</f>
-        <v/>
-      </c>
-      <c r="K18">
-        <f>IF(I4="","",I4*(1+J4/100))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="E19">
-        <f>IF(B5="","",B5*C5)</f>
-        <v/>
-      </c>
-      <c r="F19">
-        <f>IF(D5="","",B5*D5/2)</f>
-        <v/>
-      </c>
-      <c r="G19">
-        <f>IF(E5="","",E5+F5)</f>
-        <v/>
-      </c>
-      <c r="I19">
-        <f>IF(G5="","",G5-H5)</f>
-        <v/>
-      </c>
-      <c r="K19">
-        <f>IF(I5="","",I5*(1+J5/100))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="E20">
-        <f>IF(B6="","",B6*C6)</f>
-        <v/>
-      </c>
-      <c r="F20">
-        <f>IF(D6="","",B6*D6/2)</f>
-        <v/>
-      </c>
-      <c r="G20">
-        <f>IF(E6="","",E6+F6)</f>
-        <v/>
-      </c>
-      <c r="I20">
-        <f>IF(G6="","",G6-H6)</f>
-        <v/>
-      </c>
-      <c r="K20">
-        <f>IF(I6="","",I6*(1+J6/100))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="E21">
-        <f>IF(B7="","",B7*C7)</f>
-        <v/>
-      </c>
-      <c r="F21">
-        <f>IF(D7="","",B7*D7/2)</f>
-        <v/>
-      </c>
-      <c r="G21">
-        <f>IF(E7="","",E7+F7)</f>
-        <v/>
-      </c>
-      <c r="I21">
-        <f>IF(G7="","",G7-H7)</f>
-        <v/>
-      </c>
-      <c r="K21">
-        <f>IF(I7="","",I7*(1+J7/100))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="E22">
-        <f>IF(B8="","",B8*C8)</f>
-        <v/>
-      </c>
-      <c r="F22">
-        <f>IF(D8="","",B8*D8/2)</f>
-        <v/>
-      </c>
-      <c r="G22">
-        <f>IF(E8="","",E8+F8)</f>
-        <v/>
-      </c>
-      <c r="I22">
-        <f>IF(G8="","",G8-H8)</f>
-        <v/>
-      </c>
-      <c r="J22" s="43" t="inlineStr">
-        <is>
-          <t>Elevation Areas — Manual p. 21-23</t>
-        </is>
-      </c>
-      <c r="K22">
-        <f>IF(I8="","",I8*(1+J8/100))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="E23">
-        <f>IF(B9="","",B9*C9)</f>
-        <v/>
-      </c>
-      <c r="F23">
-        <f>IF(D9="","",B9*D9/2)</f>
-        <v/>
-      </c>
-      <c r="G23">
-        <f>IF(E9="","",E9+F9)</f>
-        <v/>
-      </c>
-      <c r="I23">
-        <f>IF(G9="","",G9-H9)</f>
-        <v/>
-      </c>
-      <c r="K23">
-        <f>IF(I9="","",I9*(1+J9/100))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="E24">
-        <f>IF(B10="","",B10*C10)</f>
-        <v/>
-      </c>
-      <c r="F24">
-        <f>IF(D10="","",B10*D10/2)</f>
-        <v/>
-      </c>
-      <c r="G24">
-        <f>IF(E10="","",E10+F10)</f>
-        <v/>
-      </c>
-      <c r="I24">
-        <f>IF(G10="","",G10-H10)</f>
-        <v/>
-      </c>
-      <c r="K24">
-        <f>IF(I10="","",I10*(1+J10/100))</f>
-        <v/>
       </c>
     </row>
     <row r="25">
       <c r="E25">
-        <f>IF(B11="","",B11*C11)</f>
+        <f>IF(B4="","",B4*C4)</f>
         <v/>
       </c>
       <c r="F25">
-        <f>IF(D11="","",B11*D11/2)</f>
+        <f>IF(D4="","",B4*D4/2)</f>
         <v/>
       </c>
       <c r="G25">
-        <f>IF(E11="","",E11+F11)</f>
+        <f>IF(E4="","",E4+F4)</f>
         <v/>
       </c>
       <c r="I25">
-        <f>IF(G11="","",G11-H11)</f>
+        <f>IF(G4="","",G4-H4)</f>
         <v/>
       </c>
       <c r="K25">
-        <f>IF(I11="","",I11*(1+J11/100))</f>
+        <f>IF(I4="","",I4*(1+J4/100))</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="E26">
-        <f>IF(B12="","",B12*C12)</f>
+        <f>IF(B5="","",B5*C5)</f>
         <v/>
       </c>
       <c r="F26">
-        <f>IF(D12="","",B12*D12/2)</f>
+        <f>IF(D5="","",B5*D5/2)</f>
         <v/>
       </c>
       <c r="G26">
-        <f>IF(E12="","",E12+F12)</f>
+        <f>IF(E5="","",E5+F5)</f>
         <v/>
       </c>
       <c r="I26">
-        <f>IF(G12="","",G12-H12)</f>
+        <f>IF(G5="","",G5-H5)</f>
         <v/>
       </c>
       <c r="K26">
-        <f>IF(I12="","",I12*(1+J12/100))</f>
+        <f>IF(I5="","",I5*(1+J5/100))</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="E27">
+        <f>IF(B6="","",B6*C6)</f>
+        <v/>
+      </c>
+      <c r="F27">
+        <f>IF(D6="","",B6*D6/2)</f>
+        <v/>
+      </c>
+      <c r="G27">
+        <f>IF(E6="","",E6+F6)</f>
+        <v/>
+      </c>
+      <c r="I27">
+        <f>IF(G6="","",G6-H6)</f>
+        <v/>
+      </c>
+      <c r="K27">
+        <f>IF(I6="","",I6*(1+J6/100))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="E28">
+        <f>IF(B7="","",B7*C7)</f>
+        <v/>
+      </c>
+      <c r="F28">
+        <f>IF(D7="","",B7*D7/2)</f>
+        <v/>
+      </c>
+      <c r="G28">
+        <f>IF(E7="","",E7+F7)</f>
+        <v/>
+      </c>
+      <c r="I28">
+        <f>IF(G7="","",G7-H7)</f>
+        <v/>
+      </c>
+      <c r="K28">
+        <f>IF(I7="","",I7*(1+J7/100))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="E29">
+        <f>IF(B8="","",B8*C8)</f>
+        <v/>
+      </c>
+      <c r="F29">
+        <f>IF(D8="","",B8*D8/2)</f>
+        <v/>
+      </c>
+      <c r="G29">
+        <f>IF(E8="","",E8+F8)</f>
+        <v/>
+      </c>
+      <c r="I29">
+        <f>IF(G8="","",G8-H8)</f>
+        <v/>
+      </c>
+      <c r="J29" s="43" t="inlineStr">
+        <is>
+          <t>Elevation Areas — Manual p. 21-23</t>
+        </is>
+      </c>
+      <c r="K29">
+        <f>IF(I8="","",I8*(1+J8/100))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="E30">
+        <f>IF(B9="","",B9*C9)</f>
+        <v/>
+      </c>
+      <c r="F30">
+        <f>IF(D9="","",B9*D9/2)</f>
+        <v/>
+      </c>
+      <c r="G30">
+        <f>IF(E9="","",E9+F9)</f>
+        <v/>
+      </c>
+      <c r="I30">
+        <f>IF(G9="","",G9-H9)</f>
+        <v/>
+      </c>
+      <c r="K30">
+        <f>IF(I9="","",I9*(1+J9/100))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="E31">
+        <f>IF(B10="","",B10*C10)</f>
+        <v/>
+      </c>
+      <c r="F31">
+        <f>IF(D10="","",B10*D10/2)</f>
+        <v/>
+      </c>
+      <c r="G31">
+        <f>IF(E10="","",E10+F10)</f>
+        <v/>
+      </c>
+      <c r="I31">
+        <f>IF(G10="","",G10-H10)</f>
+        <v/>
+      </c>
+      <c r="K31">
+        <f>IF(I10="","",I10*(1+J10/100))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="E32">
+        <f>IF(B11="","",B11*C11)</f>
+        <v/>
+      </c>
+      <c r="F32">
+        <f>IF(D11="","",B11*D11/2)</f>
+        <v/>
+      </c>
+      <c r="G32">
+        <f>IF(E11="","",E11+F11)</f>
+        <v/>
+      </c>
+      <c r="I32">
+        <f>IF(G11="","",G11-H11)</f>
+        <v/>
+      </c>
+      <c r="K32">
+        <f>IF(I11="","",I11*(1+J11/100))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="E33">
+        <f>IF(B12="","",B12*C12)</f>
+        <v/>
+      </c>
+      <c r="F33">
+        <f>IF(D12="","",B12*D12/2)</f>
+        <v/>
+      </c>
+      <c r="G33">
+        <f>IF(E12="","",E12+F12)</f>
+        <v/>
+      </c>
+      <c r="I33">
+        <f>IF(G12="","",G12-H12)</f>
+        <v/>
+      </c>
+      <c r="K33">
+        <f>IF(I12="","",I12*(1+J12/100))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="E34">
         <f>IF(B13="","",B13*C13)</f>
         <v/>
       </c>
-      <c r="F27">
+      <c r="F34">
         <f>IF(D13="","",B13*D13/2)</f>
         <v/>
       </c>
-      <c r="G27">
+      <c r="G34">
         <f>IF(E13="","",E13+F13)</f>
         <v/>
       </c>
-      <c r="I27">
+      <c r="I34">
         <f>IF(G13="","",G13-H13)</f>
         <v/>
       </c>
-      <c r="K27">
+      <c r="K34">
         <f>IF(I13="","",I13*(1+J13/100))</f>
         <v/>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>TOTALS</t>
-        </is>
-      </c>
-      <c r="G29" s="7">
-        <f>SUM(G4:G14)</f>
-        <v/>
-      </c>
-      <c r="H29" s="7">
-        <f>SUM(H4:H14)</f>
-        <v/>
-      </c>
-      <c r="I29" s="7">
-        <f>SUM(I4:I14)</f>
-        <v/>
-      </c>
-      <c r="K29" s="7">
-        <f>SUM(K4:K14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30"/>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL SQUARES (÷100)</t>
-        </is>
-      </c>
-      <c r="K31" s="12">
-        <f>K15/100</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32"/>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>TRIM &amp; ACCESSORIES</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>Corner Trim:</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>J-Channel:</t>
-        </is>
-      </c>
-    </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Fascia:</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>Soffit:</t>
-        </is>
-      </c>
-    </row>
+          <t>TOTALS</t>
+        </is>
+      </c>
+      <c r="G36" s="7">
+        <f>SUM(G4:G14)</f>
+        <v/>
+      </c>
+      <c r="H36" s="7">
+        <f>SUM(H4:H14)</f>
+        <v/>
+      </c>
+      <c r="I36" s="7">
+        <f>SUM(I4:I14)</f>
+        <v/>
+      </c>
+      <c r="K36" s="7">
+        <f>SUM(K4:K14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Frieze Board:</t>
-        </is>
+          <t>TOTAL SQUARES (÷100)</t>
+        </is>
+      </c>
+      <c r="K38" s="12">
+        <f>K15/100</f>
+        <v/>
       </c>
     </row>
     <row r="39"/>
     <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>TRIM &amp; ACCESSORIES</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Corner Trim:</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>J-Channel:</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Fascia:</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Soffit:</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Frieze Board:</t>
+        </is>
+      </c>
+    </row>
+    <row r="46"/>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>NOTES:</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
+    <row r="48">
+      <c r="A48" t="inlineStr">
         <is>
           <t>• Typical waste: 10% for vinyl siding, 15% for lap siding</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>• Deduct 50% for windows, 100% for doors (or calculate exact)</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>• Southeast Texas: Consider hurricane-rated fasteners</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr">
         <is>
           <t>• Order J-channel for all openings and transitions</t>
         </is>
@@ -3829,7 +4334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -3978,93 +4483,140 @@
     </row>
     <row r="14"/>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="40" t="inlineStr">
+        <is>
+          <t>STEP 5 — WINDOWS &amp; DOORS TAKEOFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>INSTRUCTIONS:</t>
+        </is>
+      </c>
+      <c r="F16" s="35" t="inlineStr">
+        <is>
+          <t>💡 TIPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="27" t="inlineStr">
+        <is>
+          <t>1. Use the window/door schedule FIRST—don't scale from plans</t>
+        </is>
+      </c>
+      <c r="F17" s="27" t="inlineStr">
+        <is>
+          <t>• Always use the schedule, not floor plan dimensions</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="27" t="inlineStr">
+        <is>
+          <t>2. Record each unit: ID, size, type, quantity</t>
+        </is>
+      </c>
+      <c r="F18" s="27" t="inlineStr">
+        <is>
+          <t>• Check for conflicting tags on elevations</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="27" t="inlineStr">
+        <is>
+          <t>3. Note special requirements: tempered, impact-rated, shapes</t>
+        </is>
+      </c>
+      <c r="F19" s="27" t="inlineStr">
+        <is>
+          <t>• Note special glass requirements</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="27" t="inlineStr">
+        <is>
+          <t>4. Verify counts by cross-checking schedule vs elevations</t>
+        </is>
+      </c>
+      <c r="F20" s="36" t="inlineStr">
+        <is>
+          <t>📖 Manual: p. 24-25 — Schedules</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>WINDOW &amp; DOOR SCHEDULE</t>
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>WINDOWS</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
         <is>
           <t>Tag</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B25" s="13" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="C18" s="13" t="inlineStr">
+      <c r="C25" s="13" t="inlineStr">
         <is>
           <t>Size (WxH)</t>
         </is>
       </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="D25" s="13" t="inlineStr">
         <is>
           <t>Rough Opening</t>
         </is>
       </c>
-      <c r="E18" s="13" t="inlineStr">
+      <c r="E25" s="13" t="inlineStr">
         <is>
           <t>Header Size</t>
         </is>
       </c>
-      <c r="F18" s="13" t="inlineStr">
+      <c r="F25" s="13" t="inlineStr">
         <is>
           <t>Type/Material</t>
         </is>
       </c>
-      <c r="G18" s="13" t="inlineStr">
+      <c r="G25" s="13" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
-      <c r="H18" s="13" t="inlineStr">
+      <c r="H25" s="13" t="inlineStr">
         <is>
           <t>Unit Price</t>
         </is>
       </c>
-    </row>
-    <row r="19">
-      <c r="H19" s="14" t="n"/>
-    </row>
-    <row r="20">
-      <c r="H20" s="14" t="n"/>
-      <c r="I20" s="43" t="inlineStr">
-        <is>
-          <t>Schedule Example — Manual p. 24-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="H21" s="14" t="n"/>
-    </row>
-    <row r="22">
-      <c r="H22" s="14" t="n"/>
-    </row>
-    <row r="23">
-      <c r="H23" s="14" t="n"/>
-    </row>
-    <row r="24">
-      <c r="H24" s="14" t="n"/>
-    </row>
-    <row r="25">
-      <c r="H25" s="14" t="n"/>
     </row>
     <row r="26">
       <c r="H26" s="14" t="n"/>
     </row>
     <row r="27">
       <c r="H27" s="14" t="n"/>
+      <c r="I27" s="43" t="inlineStr">
+        <is>
+          <t>Schedule Example — Manual p. 24-25</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="H28" s="14" t="n"/>
@@ -4084,55 +4636,14 @@
     <row r="33">
       <c r="H33" s="14" t="n"/>
     </row>
-    <row r="34"/>
+    <row r="34">
+      <c r="H34" s="14" t="n"/>
+    </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>DOORS</t>
-        </is>
-      </c>
+      <c r="H35" s="14" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="15" t="inlineStr">
-        <is>
-          <t>Tag</t>
-        </is>
-      </c>
-      <c r="B36" s="15" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="C36" s="15" t="inlineStr">
-        <is>
-          <t>Size (WxH)</t>
-        </is>
-      </c>
-      <c r="D36" s="15" t="inlineStr">
-        <is>
-          <t>Rough Opening</t>
-        </is>
-      </c>
-      <c r="E36" s="15" t="inlineStr">
-        <is>
-          <t>Header Size</t>
-        </is>
-      </c>
-      <c r="F36" s="15" t="inlineStr">
-        <is>
-          <t>Type/Material</t>
-        </is>
-      </c>
-      <c r="G36" s="15" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="H36" s="15" t="inlineStr">
-        <is>
-          <t>Unit Price</t>
-        </is>
-      </c>
+      <c r="H36" s="14" t="n"/>
     </row>
     <row r="37">
       <c r="H37" s="14" t="n"/>
@@ -4146,14 +4657,55 @@
     <row r="40">
       <c r="H40" s="14" t="n"/>
     </row>
-    <row r="41">
-      <c r="H41" s="14" t="n"/>
-    </row>
+    <row r="41"/>
     <row r="42">
-      <c r="H42" s="14" t="n"/>
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>DOORS</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="H43" s="14" t="n"/>
+      <c r="A43" s="15" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="B43" s="15" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="C43" s="15" t="inlineStr">
+        <is>
+          <t>Size (WxH)</t>
+        </is>
+      </c>
+      <c r="D43" s="15" t="inlineStr">
+        <is>
+          <t>Rough Opening</t>
+        </is>
+      </c>
+      <c r="E43" s="15" t="inlineStr">
+        <is>
+          <t>Header Size</t>
+        </is>
+      </c>
+      <c r="F43" s="15" t="inlineStr">
+        <is>
+          <t>Type/Material</t>
+        </is>
+      </c>
+      <c r="G43" s="15" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="H43" s="15" t="inlineStr">
+        <is>
+          <t>Unit Price</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="H44" s="14" t="n"/>
@@ -4179,30 +4731,51 @@
     <row r="51">
       <c r="H51" s="14" t="n"/>
     </row>
-    <row r="52"/>
+    <row r="52">
+      <c r="H52" s="14" t="n"/>
+    </row>
     <row r="53">
-      <c r="A53" s="3" t="inlineStr">
+      <c r="H53" s="14" t="n"/>
+    </row>
+    <row r="54">
+      <c r="H54" s="14" t="n"/>
+    </row>
+    <row r="55">
+      <c r="H55" s="14" t="n"/>
+    </row>
+    <row r="56">
+      <c r="H56" s="14" t="n"/>
+    </row>
+    <row r="57">
+      <c r="H57" s="14" t="n"/>
+    </row>
+    <row r="58">
+      <c r="H58" s="14" t="n"/>
+    </row>
+    <row r="59"/>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
+      <c r="G60" t="inlineStr">
         <is>
           <t>Window Count:</t>
         </is>
       </c>
-      <c r="H53">
+      <c r="H60">
         <f>SUM(B5:B19)</f>
         <v/>
       </c>
     </row>
-    <row r="54">
-      <c r="G54" t="inlineStr">
+    <row r="61">
+      <c r="G61" t="inlineStr">
         <is>
           <t>Door Count:</t>
         </is>
       </c>
-      <c r="H54">
+      <c r="H61">
         <f>SUM(B23:B37)</f>
         <v/>
       </c>
@@ -4232,7 +4805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4385,331 +4958,229 @@
     </row>
     <row r="22"/>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
+      <c r="A23" s="41" t="inlineStr">
+        <is>
+          <t>STEP 6 — FINAL MATERIAL SUMMARY (READY TO QUOTE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="30" t="inlineStr">
+        <is>
+          <t>COMPLETION CHECKLIST:</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="32" t="inlineStr">
+        <is>
+          <t>☐ Foundation sheet completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="32" t="inlineStr">
+        <is>
+          <t>☐ Wall framing sheet completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="32" t="inlineStr">
+        <is>
+          <t>☐ Roof sheet completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="32" t="inlineStr">
+        <is>
+          <t>☐ Siding &amp; exterior sheet completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="32" t="inlineStr">
+        <is>
+          <t>☐ Windows &amp; doors sheet completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="32" t="inlineStr">
+        <is>
+          <t>☐ All assumptions noted for customer/engineer review</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="42" t="inlineStr">
+        <is>
+          <t>✅ When complete, this summary is ready to key into the quoting system</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="36" t="inlineStr">
+        <is>
+          <t>📖 See Manual: p. 26-27 — Complete Example &amp; Final Checks</t>
+        </is>
+      </c>
+    </row>
+    <row r="33"/>
+    <row r="34">
+      <c r="A34" s="16" t="inlineStr">
         <is>
           <t>MATERIAL SUMMARY - READY TO QUOTE</t>
         </is>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Project:</t>
-        </is>
-      </c>
-      <c r="B25">
-        <f>'Project Info'!B4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Job Number:</t>
-        </is>
-      </c>
-      <c r="B26">
-        <f>'Project Info'!B5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27"/>
-    <row r="28">
-      <c r="A28" s="17" t="inlineStr">
-        <is>
-          <t>FRAMING LUMBER</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="18" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="B29" s="18" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="C29" s="18" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="D29" s="18" t="inlineStr">
-        <is>
-          <t>Unit Price</t>
-        </is>
-      </c>
-      <c r="E29" s="18" t="inlineStr">
-        <is>
-          <t>Extended</t>
-        </is>
-      </c>
-      <c r="F29" s="18" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>2x4x8 Studs</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>2x6x8 Studs</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>EA</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="n"/>
-      <c r="D31" s="14" t="n"/>
-      <c r="E31" s="14">
-        <f>C9*D9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>2x4 Plates (Treated)</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="n"/>
-      <c r="D32" s="14" t="n"/>
-      <c r="E32" s="14">
-        <f>C10*D10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>2x6 Plates (Treated)</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="n"/>
-      <c r="D33" s="14" t="n"/>
-      <c r="E33" s="14">
-        <f>C11*D11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>2x4 Top Plates</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="n"/>
-      <c r="D34" s="14" t="n"/>
-      <c r="E34" s="14">
-        <f>C12*D12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>2x6 Top Plates</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="n"/>
-      <c r="D35" s="14" t="n"/>
-      <c r="E35" s="14">
-        <f>C13*D13</f>
-        <v/>
-      </c>
-    </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2x6 Headers</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="n"/>
-      <c r="D36" s="14" t="n"/>
-      <c r="E36" s="14">
-        <f>C14*D14</f>
+          <t>Project:</t>
+        </is>
+      </c>
+      <c r="B36">
+        <f>'Project Info'!B4</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2x8 Headers</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="n"/>
-      <c r="D37" s="14" t="n"/>
-      <c r="E37" s="14">
-        <f>C15*D15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>2x10 Headers</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="n"/>
-      <c r="D38" s="14" t="n"/>
-      <c r="E38" s="14">
-        <f>C16*D16</f>
-        <v/>
-      </c>
-    </row>
+          <t>Job Number:</t>
+        </is>
+      </c>
+      <c r="B37">
+        <f>'Project Info'!B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38"/>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>2x12 Headers</t>
-        </is>
-      </c>
-    </row>
-    <row r="40"/>
+      <c r="A39" s="17" t="inlineStr">
+        <is>
+          <t>FRAMING LUMBER</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="18" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B40" s="18" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="C40" s="18" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="D40" s="18" t="inlineStr">
+        <is>
+          <t>Unit Price</t>
+        </is>
+      </c>
+      <c r="E40" s="18" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
+      </c>
+      <c r="F40" s="18" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
     <row r="41">
-      <c r="A41" s="17" t="inlineStr">
-        <is>
-          <t>ROOF MATERIALS</t>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2x4x8 Studs</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="18" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="B42" s="18" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="C42" s="18" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="D42" s="18" t="inlineStr">
-        <is>
-          <t>Unit Price</t>
-        </is>
-      </c>
-      <c r="E42" s="18" t="inlineStr">
-        <is>
-          <t>Extended</t>
-        </is>
-      </c>
-      <c r="F42" s="18" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2x6x8 Studs</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="n"/>
+      <c r="D42" s="14" t="n"/>
+      <c r="E42" s="14">
+        <f>C9*D9</f>
+        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>7/16" OSB Sheathing</t>
+          <t>2x4 Plates (Treated)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Sheets</t>
+          <t>LF</t>
         </is>
       </c>
       <c r="C43" s="4" t="n"/>
       <c r="D43" s="14" t="n"/>
       <c r="E43" s="14">
-        <f>C21*D21</f>
+        <f>C10*D10</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Shingles (Architectural)</t>
+          <t>2x6 Plates (Treated)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Bundles</t>
+          <t>LF</t>
         </is>
       </c>
       <c r="C44" s="4" t="n"/>
       <c r="D44" s="14" t="n"/>
       <c r="E44" s="14">
-        <f>C22*D22</f>
+        <f>C11*D11</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Hip &amp; Ridge Cap</t>
+          <t>2x4 Top Plates</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Bundles</t>
+          <t>LF</t>
         </is>
       </c>
       <c r="C45" s="4" t="n"/>
       <c r="D45" s="14" t="n"/>
       <c r="E45" s="14">
-        <f>C23*D23</f>
+        <f>C12*D12</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Starter Strip</t>
+          <t>2x6 Top Plates</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -4720,303 +5191,465 @@
       <c r="C46" s="4" t="n"/>
       <c r="D46" s="14" t="n"/>
       <c r="E46" s="14">
-        <f>C24*D24</f>
+        <f>C13*D13</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Drip Edge</t>
+          <t>2x6 Headers</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Felt/Underlayment</t>
+          <t>2x8 Headers</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Rolls</t>
+          <t>LF</t>
         </is>
       </c>
       <c r="C48" s="4" t="n"/>
       <c r="D48" s="14" t="n"/>
       <c r="E48" s="14">
-        <f>C26*D26</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49"/>
+        <f>C15*D15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2x10 Headers</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>LF</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="n"/>
+      <c r="D49" s="14" t="n"/>
+      <c r="E49" s="14">
+        <f>C16*D16</f>
+        <v/>
+      </c>
+    </row>
     <row r="50">
-      <c r="A50" s="17" t="inlineStr">
-        <is>
-          <t>FOUNDATION</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="18" t="inlineStr">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2x12 Headers</t>
+        </is>
+      </c>
+    </row>
+    <row r="51"/>
+    <row r="52">
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t>ROOF MATERIALS</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="18" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="B51" s="18" t="inlineStr">
+      <c r="B53" s="18" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="C51" s="18" t="inlineStr">
+      <c r="C53" s="18" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="D51" s="18" t="inlineStr">
+      <c r="D53" s="18" t="inlineStr">
         <is>
           <t>Unit Price</t>
         </is>
       </c>
-      <c r="E51" s="18" t="inlineStr">
+      <c r="E53" s="18" t="inlineStr">
         <is>
           <t>Extended</t>
         </is>
       </c>
-      <c r="F51" s="18" t="inlineStr">
+      <c r="F53" s="18" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Concrete 3000 PSI</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>CY</t>
-        </is>
-      </c>
-      <c r="C52" s="4" t="n"/>
-      <c r="D52" s="14" t="n"/>
-      <c r="E52" s="14">
-        <f>C30*D30</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>#3 Rebar</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="C53" s="4" t="n"/>
-      <c r="D53" s="14" t="n"/>
-      <c r="E53" s="14">
-        <f>C31*D31</f>
-        <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>#4 Rebar</t>
+          <t>7/16" OSB Sheathing</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>LF</t>
+          <t>Sheets</t>
         </is>
       </c>
       <c r="C54" s="4" t="n"/>
       <c r="D54" s="14" t="n"/>
       <c r="E54" s="14">
-        <f>C32*D32</f>
+        <f>C21*D21</f>
         <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>6mil Vapor Barrier</t>
+          <t>Shingles (Architectural)</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>Bundles</t>
         </is>
       </c>
       <c r="C55" s="4" t="n"/>
       <c r="D55" s="14" t="n"/>
       <c r="E55" s="14">
-        <f>C33*D33</f>
+        <f>C22*D22</f>
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Anchor Bolts</t>
+          <t>Hip &amp; Ridge Cap</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>EA</t>
+          <t>Bundles</t>
         </is>
       </c>
       <c r="C56" s="4" t="n"/>
       <c r="D56" s="14" t="n"/>
       <c r="E56" s="14">
-        <f>C34*D34</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57"/>
+        <f>C23*D23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Starter Strip</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>LF</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="n"/>
+      <c r="D57" s="14" t="n"/>
+      <c r="E57" s="14">
+        <f>C24*D24</f>
+        <v/>
+      </c>
+    </row>
     <row r="58">
-      <c r="A58" s="17" t="inlineStr">
-        <is>
-          <t>EXTERIOR FINISHES</t>
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Drip Edge</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="18" t="inlineStr">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Felt/Underlayment</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Rolls</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="n"/>
+      <c r="D59" s="14" t="n"/>
+      <c r="E59" s="14">
+        <f>C26*D26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60"/>
+    <row r="61">
+      <c r="A61" s="17" t="inlineStr">
+        <is>
+          <t>FOUNDATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="18" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="B59" s="18" t="inlineStr">
+      <c r="B62" s="18" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="C59" s="18" t="inlineStr">
+      <c r="C62" s="18" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="D59" s="18" t="inlineStr">
+      <c r="D62" s="18" t="inlineStr">
         <is>
           <t>Unit Price</t>
         </is>
       </c>
-      <c r="E59" s="18" t="inlineStr">
+      <c r="E62" s="18" t="inlineStr">
         <is>
           <t>Extended</t>
         </is>
       </c>
-      <c r="F59" s="18" t="inlineStr">
+      <c r="F62" s="18" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Siding</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Squares</t>
-        </is>
-      </c>
-      <c r="C60" s="4" t="n"/>
-      <c r="D60" s="14" t="n"/>
-      <c r="E60" s="14">
-        <f>C38*D38</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>J-Channel</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="C61" s="4" t="n"/>
-      <c r="D61" s="14" t="n"/>
-      <c r="E61" s="14">
-        <f>C39*D39</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Corner Trim</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>EA</t>
-        </is>
-      </c>
-      <c r="C62" s="4" t="n"/>
-      <c r="D62" s="14" t="n"/>
-      <c r="E62" s="14">
-        <f>C40*D40</f>
-        <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Fascia</t>
+          <t>Concrete 3000 PSI</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>LF</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="C63" s="4" t="n"/>
       <c r="D63" s="14" t="n"/>
       <c r="E63" s="14">
-        <f>C41*D41</f>
+        <f>C30*D30</f>
         <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Soffit</t>
+          <t>#3 Rebar</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>LF</t>
         </is>
       </c>
       <c r="C64" s="4" t="n"/>
       <c r="D64" s="14" t="n"/>
       <c r="E64" s="14">
+        <f>C31*D31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>#4 Rebar</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>LF</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="n"/>
+      <c r="D65" s="14" t="n"/>
+      <c r="E65" s="14">
+        <f>C32*D32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>6mil Vapor Barrier</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="n"/>
+      <c r="D66" s="14" t="n"/>
+      <c r="E66" s="14">
+        <f>C33*D33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Anchor Bolts</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="n"/>
+      <c r="D67" s="14" t="n"/>
+      <c r="E67" s="14">
+        <f>C34*D34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68"/>
+    <row r="69">
+      <c r="A69" s="17" t="inlineStr">
+        <is>
+          <t>EXTERIOR FINISHES</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="18" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B70" s="18" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="C70" s="18" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="D70" s="18" t="inlineStr">
+        <is>
+          <t>Unit Price</t>
+        </is>
+      </c>
+      <c r="E70" s="18" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
+      </c>
+      <c r="F70" s="18" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Siding</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Squares</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="n"/>
+      <c r="D71" s="14" t="n"/>
+      <c r="E71" s="14">
+        <f>C38*D38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>J-Channel</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>LF</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="n"/>
+      <c r="D72" s="14" t="n"/>
+      <c r="E72" s="14">
+        <f>C39*D39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Corner Trim</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="n"/>
+      <c r="D73" s="14" t="n"/>
+      <c r="E73" s="14">
+        <f>C40*D40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Fascia</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>LF</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="n"/>
+      <c r="D74" s="14" t="n"/>
+      <c r="E74" s="14">
+        <f>C41*D41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Soffit</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="n"/>
+      <c r="D75" s="14" t="n"/>
+      <c r="E75" s="14">
         <f>C42*D42</f>
         <v/>
       </c>
     </row>
-    <row r="65"/>
-    <row r="66">
-      <c r="D66" s="19" t="inlineStr">
+    <row r="76"/>
+    <row r="77">
+      <c r="D77" s="19" t="inlineStr">
         <is>
           <t>GRAND TOTAL:</t>
         </is>
       </c>
-      <c r="E66" s="20" t="n"/>
+      <c r="E77" s="20" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>

<commit_message>
Fix diagram readability and double image sizes in Excel workbook
Co-authored-by: lancejlene-oss <240118005+lancejlene-oss@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/templates/worksheet.xlsx
+++ b/templates/worksheet.xlsx
@@ -381,10 +381,10 @@
     <from>
       <col>3</col>
       <colOff>0</colOff>
-      <row>2</row>
+      <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="2000250"/>
+    <ext cx="6667500" cy="5000625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -411,10 +411,10 @@
     <from>
       <col>13</col>
       <colOff>0</colOff>
-      <row>2</row>
+      <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="2333625"/>
+    <ext cx="6667500" cy="5829300"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -441,10 +441,10 @@
     <from>
       <col>15</col>
       <colOff>0</colOff>
-      <row>2</row>
+      <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="2076450"/>
+    <ext cx="6667500" cy="5181600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -471,10 +471,10 @@
     <from>
       <col>3</col>
       <colOff>0</colOff>
-      <row>2</row>
+      <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1924050"/>
+    <ext cx="6667500" cy="4819650"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -501,10 +501,10 @@
     <from>
       <col>11</col>
       <colOff>0</colOff>
-      <row>2</row>
+      <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="2000250"/>
+    <ext cx="6667500" cy="5000625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -531,10 +531,10 @@
     <from>
       <col>9</col>
       <colOff>0</colOff>
-      <row>2</row>
+      <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1781175"/>
+    <ext cx="6667500" cy="4448175"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -1224,7 +1224,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
@@ -1304,7 +1303,6 @@
       </c>
       <c r="B22" s="4" t="n"/>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
@@ -1360,7 +1358,6 @@
       </c>
       <c r="B30" s="4" t="n"/>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
@@ -1514,7 +1511,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
@@ -1961,7 +1957,6 @@
         <v/>
       </c>
     </row>
-    <row r="34"/>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
@@ -2115,7 +2110,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
@@ -2479,7 +2473,6 @@
         <v/>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="D25" s="3" t="inlineStr">
         <is>
@@ -2503,7 +2496,6 @@
         <v/>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="D27" s="8" t="inlineStr">
         <is>
@@ -2644,7 +2636,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
@@ -2739,7 +2730,6 @@
         <v/>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
@@ -2854,7 +2844,6 @@
         <v/>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
@@ -2877,7 +2866,6 @@
         <v/>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
@@ -3029,7 +3017,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
@@ -3307,7 +3294,6 @@
         <v/>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
@@ -3331,7 +3317,6 @@
         <v/>
       </c>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
@@ -3343,7 +3328,6 @@
         <v/>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
@@ -3386,7 +3370,6 @@
         </is>
       </c>
     </row>
-    <row r="34"/>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
@@ -3528,7 +3511,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
@@ -3623,7 +3605,6 @@
     <row r="28">
       <c r="H28" s="14" t="n"/>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
@@ -3718,7 +3699,6 @@
     <row r="46">
       <c r="H46" s="14" t="n"/>
     </row>
-    <row r="47"/>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
@@ -3847,7 +3827,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -3870,7 +3849,6 @@
         <v/>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="17" t="inlineStr">
         <is>
@@ -4090,7 +4068,6 @@
         <v/>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
         <is>
@@ -4238,7 +4215,6 @@
         <v/>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="17" t="inlineStr">
         <is>
@@ -4368,7 +4344,6 @@
         <v/>
       </c>
     </row>
-    <row r="47"/>
     <row r="48">
       <c r="A48" s="17" t="inlineStr">
         <is>
@@ -4498,7 +4473,6 @@
         <v/>
       </c>
     </row>
-    <row r="55"/>
     <row r="56">
       <c r="D56" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix overlapping text in roof and foundation diagrams
Co-authored-by: lancejlene-oss <240118005+lancejlene-oss@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/templates/worksheet.xlsx
+++ b/templates/worksheet.xlsx
@@ -398,6 +398,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -428,6 +431,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -518,6 +524,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -548,6 +557,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>

</xml_diff>